<commit_message>
initial refinement run with Germany 2024 data
</commit_message>
<xml_diff>
--- a/Supporting files/Indicators.xlsx
+++ b/Supporting files/Indicators.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="497" uniqueCount="321">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="498" uniqueCount="322">
   <si>
     <t xml:space="preserve">Country</t>
   </si>
@@ -989,6 +989,9 @@
   </si>
   <si>
     <t xml:space="preserve">-</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Disaster coping capacity</t>
   </si>
 </sst>
 </file>
@@ -1076,7 +1079,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1102,10 +1105,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1135,7 +1134,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:K210"/>
-  <sheetFormatPr defaultColWidth="11.2421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.2578125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10.67"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="10.44"/>
@@ -5763,7 +5762,9 @@
       <c r="I132" s="1" t="n">
         <v>0.656</v>
       </c>
-      <c r="J132" s="7"/>
+      <c r="J132" s="3" t="n">
+        <v>2.1</v>
+      </c>
       <c r="K132" s="6" t="n">
         <v>1.2156</v>
       </c>
@@ -8515,7 +8516,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F36"/>
-  <sheetFormatPr defaultColWidth="11.2421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.2578125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10.67"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16.33"/>
@@ -8768,7 +8769,7 @@
       <c r="A13" s="4" t="s">
         <v>237</v>
       </c>
-      <c r="B13" s="8" t="n">
+      <c r="B13" s="7" t="n">
         <v>30.6</v>
       </c>
       <c r="C13" s="1" t="n">
@@ -9261,7 +9262,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultColWidth="11.2421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.2578125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="1" style="0" width="10.67"/>
   </cols>
@@ -9323,7 +9324,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C37"/>
-  <sheetFormatPr defaultColWidth="11.2421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.2578125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="1" style="0" width="10.67"/>
   </cols>
@@ -9752,7 +9753,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:BU36"/>
-  <sheetFormatPr defaultColWidth="11.2421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.2578125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="73" min="1" style="0" width="10.67"/>
   </cols>
@@ -17715,7 +17716,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E25"/>
-  <sheetFormatPr defaultColWidth="11.2421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.2578125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="1" style="0" width="10.67"/>
   </cols>
@@ -17741,16 +17742,16 @@
       <c r="A2" s="1" t="s">
         <v>281</v>
       </c>
-      <c r="B2" s="9" t="n">
+      <c r="B2" s="8" t="n">
         <v>6146</v>
       </c>
-      <c r="C2" s="9" t="n">
+      <c r="C2" s="8" t="n">
         <v>767220</v>
       </c>
-      <c r="D2" s="9" t="n">
+      <c r="D2" s="8" t="n">
         <v>223897448</v>
       </c>
-      <c r="E2" s="9" t="n">
+      <c r="E2" s="8" t="n">
         <v>47369357</v>
       </c>
     </row>
@@ -17761,13 +17762,13 @@
       <c r="B3" s="2" t="n">
         <v>844</v>
       </c>
-      <c r="C3" s="9" t="n">
+      <c r="C3" s="8" t="n">
         <v>99529</v>
       </c>
-      <c r="D3" s="9" t="n">
+      <c r="D3" s="8" t="n">
         <v>52181098</v>
       </c>
-      <c r="E3" s="9" t="n">
+      <c r="E3" s="8" t="n">
         <v>22775597</v>
       </c>
     </row>
@@ -17778,13 +17779,13 @@
       <c r="B4" s="2" t="n">
         <v>851</v>
       </c>
-      <c r="C4" s="9" t="n">
+      <c r="C4" s="8" t="n">
         <v>83039</v>
       </c>
-      <c r="D4" s="9" t="n">
+      <c r="D4" s="8" t="n">
         <v>19576142</v>
       </c>
-      <c r="E4" s="9" t="n">
+      <c r="E4" s="8" t="n">
         <v>6245331</v>
       </c>
     </row>
@@ -17792,16 +17793,16 @@
       <c r="A5" s="1" t="s">
         <v>284</v>
       </c>
-      <c r="B5" s="9" t="n">
+      <c r="B5" s="8" t="n">
         <v>1136</v>
       </c>
-      <c r="C5" s="9" t="n">
+      <c r="C5" s="8" t="n">
         <v>90370</v>
       </c>
-      <c r="D5" s="9" t="n">
+      <c r="D5" s="8" t="n">
         <v>24641046</v>
       </c>
-      <c r="E5" s="9" t="n">
+      <c r="E5" s="8" t="n">
         <v>6594191</v>
       </c>
     </row>
@@ -17809,16 +17810,16 @@
       <c r="A6" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="B6" s="9" t="n">
+      <c r="B6" s="8" t="n">
         <v>1019</v>
       </c>
-      <c r="C6" s="9" t="n">
+      <c r="C6" s="8" t="n">
         <v>89330</v>
       </c>
-      <c r="D6" s="9" t="n">
+      <c r="D6" s="8" t="n">
         <v>17735937</v>
       </c>
-      <c r="E6" s="9" t="n">
+      <c r="E6" s="8" t="n">
         <v>5917123</v>
       </c>
     </row>
@@ -17829,13 +17830,13 @@
       <c r="B7" s="2" t="n">
         <v>751</v>
       </c>
-      <c r="C7" s="9" t="n">
+      <c r="C7" s="8" t="n">
         <v>123947</v>
       </c>
-      <c r="D7" s="9" t="n">
+      <c r="D7" s="8" t="n">
         <v>44551407</v>
       </c>
-      <c r="E7" s="9" t="n">
+      <c r="E7" s="8" t="n">
         <v>11266123</v>
       </c>
     </row>
@@ -17843,16 +17844,16 @@
       <c r="A8" s="1" t="s">
         <v>287</v>
       </c>
-      <c r="B8" s="9" t="n">
+      <c r="B8" s="8" t="n">
         <v>1103</v>
       </c>
-      <c r="C8" s="9" t="n">
+      <c r="C8" s="8" t="n">
         <v>84217</v>
       </c>
-      <c r="D8" s="9" t="n">
+      <c r="D8" s="8" t="n">
         <v>12300578</v>
       </c>
-      <c r="E8" s="9" t="n">
+      <c r="E8" s="8" t="n">
         <v>4610177</v>
       </c>
     </row>
@@ -17860,16 +17861,16 @@
       <c r="A9" s="1" t="s">
         <v>288</v>
       </c>
-      <c r="B9" s="9" t="n">
+      <c r="B9" s="8" t="n">
         <v>1705</v>
       </c>
-      <c r="C9" s="9" t="n">
+      <c r="C9" s="8" t="n">
         <v>494001</v>
       </c>
-      <c r="D9" s="9" t="n">
+      <c r="D9" s="8" t="n">
         <v>241896459</v>
       </c>
-      <c r="E9" s="9" t="n">
+      <c r="E9" s="8" t="n">
         <v>62663807</v>
       </c>
     </row>
@@ -17880,13 +17881,13 @@
       <c r="B10" s="2" t="n">
         <v>53</v>
       </c>
-      <c r="C10" s="9" t="n">
+      <c r="C10" s="8" t="n">
         <v>20730</v>
       </c>
-      <c r="D10" s="9" t="n">
+      <c r="D10" s="8" t="n">
         <v>102506980</v>
       </c>
-      <c r="E10" s="9" t="n">
+      <c r="E10" s="8" t="n">
         <v>39185116</v>
       </c>
     </row>
@@ -17894,16 +17895,16 @@
       <c r="A11" s="1" t="s">
         <v>290</v>
       </c>
-      <c r="B11" s="9" t="n">
+      <c r="B11" s="8" t="n">
         <v>2742</v>
       </c>
-      <c r="C11" s="9" t="n">
+      <c r="C11" s="8" t="n">
         <v>317975</v>
       </c>
-      <c r="D11" s="9" t="n">
+      <c r="D11" s="8" t="n">
         <v>73371263</v>
       </c>
-      <c r="E11" s="9" t="n">
+      <c r="E11" s="8" t="n">
         <v>24559442</v>
       </c>
     </row>
@@ -17914,13 +17915,13 @@
       <c r="B12" s="2" t="n">
         <v>285</v>
       </c>
-      <c r="C12" s="9" t="n">
+      <c r="C12" s="8" t="n">
         <v>66465</v>
       </c>
-      <c r="D12" s="9" t="n">
+      <c r="D12" s="8" t="n">
         <v>20488964</v>
       </c>
-      <c r="E12" s="9" t="n">
+      <c r="E12" s="8" t="n">
         <v>5587892</v>
       </c>
     </row>
@@ -17931,13 +17932,13 @@
       <c r="B13" s="2" t="n">
         <v>106</v>
       </c>
-      <c r="C13" s="9" t="n">
+      <c r="C13" s="8" t="n">
         <v>13730</v>
       </c>
-      <c r="D13" s="9" t="n">
+      <c r="D13" s="8" t="n">
         <v>3021648</v>
       </c>
-      <c r="E13" s="9" t="n">
+      <c r="E13" s="8" t="n">
         <v>911863</v>
       </c>
     </row>
@@ -17945,16 +17946,16 @@
       <c r="A14" s="1" t="s">
         <v>293</v>
       </c>
-      <c r="B14" s="9" t="n">
+      <c r="B14" s="8" t="n">
         <v>1529</v>
       </c>
-      <c r="C14" s="9" t="n">
+      <c r="C14" s="8" t="n">
         <v>193059</v>
       </c>
-      <c r="D14" s="9" t="n">
+      <c r="D14" s="8" t="n">
         <v>53000062</v>
       </c>
-      <c r="E14" s="9" t="n">
+      <c r="E14" s="8" t="n">
         <v>17745672</v>
       </c>
     </row>
@@ -17965,13 +17966,13 @@
       <c r="B15" s="2" t="n">
         <v>708</v>
       </c>
-      <c r="C15" s="9" t="n">
+      <c r="C15" s="8" t="n">
         <v>175869</v>
       </c>
-      <c r="D15" s="9" t="n">
+      <c r="D15" s="8" t="n">
         <v>71037351</v>
       </c>
-      <c r="E15" s="9" t="n">
+      <c r="E15" s="8" t="n">
         <v>12348972</v>
       </c>
     </row>
@@ -17982,13 +17983,13 @@
       <c r="B16" s="2" t="n">
         <v>202</v>
       </c>
-      <c r="C16" s="9" t="n">
+      <c r="C16" s="8" t="n">
         <v>60773</v>
       </c>
-      <c r="D16" s="9" t="n">
+      <c r="D16" s="8" t="n">
         <v>60383899</v>
       </c>
-      <c r="E16" s="9" t="n">
+      <c r="E16" s="8" t="n">
         <v>7970421</v>
       </c>
     </row>
@@ -17996,16 +17997,16 @@
       <c r="A17" s="1" t="s">
         <v>296</v>
       </c>
-      <c r="B17" s="9" t="n">
+      <c r="B17" s="8" t="n">
         <v>8189</v>
       </c>
-      <c r="C17" s="9" t="n">
+      <c r="C17" s="8" t="n">
         <v>671683</v>
       </c>
-      <c r="D17" s="9" t="n">
+      <c r="D17" s="8" t="n">
         <v>136653722</v>
       </c>
-      <c r="E17" s="9" t="n">
+      <c r="E17" s="8" t="n">
         <v>50753970</v>
       </c>
     </row>
@@ -18013,16 +18014,16 @@
       <c r="A18" s="1" t="s">
         <v>297</v>
       </c>
-      <c r="B18" s="9" t="n">
+      <c r="B18" s="8" t="n">
         <v>2922</v>
       </c>
-      <c r="C18" s="9" t="n">
+      <c r="C18" s="8" t="n">
         <v>690376</v>
       </c>
-      <c r="D18" s="9" t="n">
+      <c r="D18" s="8" t="n">
         <v>214187043</v>
       </c>
-      <c r="E18" s="9" t="n">
+      <c r="E18" s="8" t="n">
         <v>72513015</v>
       </c>
     </row>
@@ -18033,13 +18034,13 @@
       <c r="B19" s="2" t="n">
         <v>888</v>
       </c>
-      <c r="C19" s="9" t="n">
+      <c r="C19" s="8" t="n">
         <v>152219</v>
       </c>
-      <c r="D19" s="9" t="n">
+      <c r="D19" s="8" t="n">
         <v>42284530</v>
       </c>
-      <c r="E19" s="9" t="n">
+      <c r="E19" s="8" t="n">
         <v>13955965</v>
       </c>
     </row>
@@ -18047,16 +18048,16 @@
       <c r="A20" s="1" t="s">
         <v>299</v>
       </c>
-      <c r="B20" s="9" t="n">
+      <c r="B20" s="8" t="n">
         <v>1975</v>
       </c>
-      <c r="C20" s="9" t="n">
+      <c r="C20" s="8" t="n">
         <v>275433</v>
       </c>
-      <c r="D20" s="9" t="n">
+      <c r="D20" s="8" t="n">
         <v>72842820</v>
       </c>
-      <c r="E20" s="9" t="n">
+      <c r="E20" s="8" t="n">
         <v>25577398</v>
       </c>
     </row>
@@ -18067,13 +18068,13 @@
       <c r="B21" s="2" t="n">
         <v>557</v>
       </c>
-      <c r="C21" s="9" t="n">
+      <c r="C21" s="8" t="n">
         <v>94969</v>
       </c>
-      <c r="D21" s="9" t="n">
+      <c r="D21" s="8" t="n">
         <v>33737366</v>
       </c>
-      <c r="E21" s="9" t="n">
+      <c r="E21" s="8" t="n">
         <v>11720234</v>
       </c>
     </row>
@@ -18081,16 +18082,16 @@
       <c r="A22" s="1" t="s">
         <v>301</v>
       </c>
-      <c r="B22" s="9" t="n">
+      <c r="B22" s="8" t="n">
         <v>2120</v>
       </c>
-      <c r="C22" s="9" t="n">
+      <c r="C22" s="8" t="n">
         <v>453706</v>
       </c>
-      <c r="D22" s="9" t="n">
+      <c r="D22" s="8" t="n">
         <v>129317166</v>
       </c>
-      <c r="E22" s="9" t="n">
+      <c r="E22" s="8" t="n">
         <v>40566069</v>
       </c>
     </row>
@@ -18098,16 +18099,16 @@
       <c r="A23" s="1" t="s">
         <v>302</v>
       </c>
-      <c r="B23" s="9" t="n">
+      <c r="B23" s="8" t="n">
         <v>1509</v>
       </c>
-      <c r="C23" s="9" t="n">
+      <c r="C23" s="8" t="n">
         <v>256962</v>
       </c>
-      <c r="D23" s="9" t="n">
+      <c r="D23" s="8" t="n">
         <v>74314186</v>
       </c>
-      <c r="E23" s="9" t="n">
+      <c r="E23" s="8" t="n">
         <v>28208514</v>
       </c>
     </row>
@@ -18115,16 +18116,16 @@
       <c r="A24" s="1" t="s">
         <v>303</v>
       </c>
-      <c r="B24" s="9" t="n">
+      <c r="B24" s="8" t="n">
         <v>1463</v>
       </c>
-      <c r="C24" s="9" t="n">
+      <c r="C24" s="8" t="n">
         <v>953340</v>
       </c>
-      <c r="D24" s="9" t="n">
+      <c r="D24" s="8" t="n">
         <v>670994222</v>
       </c>
-      <c r="E24" s="9" t="n">
+      <c r="E24" s="8" t="n">
         <v>135397753</v>
       </c>
     </row>
@@ -18132,16 +18133,16 @@
       <c r="A25" s="1" t="s">
         <v>304</v>
       </c>
-      <c r="B25" s="9" t="n">
+      <c r="B25" s="8" t="n">
         <v>38803</v>
       </c>
-      <c r="C25" s="9" t="n">
+      <c r="C25" s="8" t="n">
         <v>6228942</v>
       </c>
-      <c r="D25" s="9" t="n">
+      <c r="D25" s="8" t="n">
         <v>2394921337</v>
       </c>
-      <c r="E25" s="9" t="n">
+      <c r="E25" s="8" t="n">
         <v>654444002</v>
       </c>
     </row>
@@ -18161,8 +18162,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultColWidth="11.2421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr defaultColWidth="11.2578125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="1" style="0" width="10.67"/>
   </cols>
@@ -18276,6 +18277,14 @@
       </c>
       <c r="C11" s="4" t="n">
         <v>0.25</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="0" t="s">
+        <v>321</v>
+      </c>
+      <c r="C12" s="0" t="n">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>